<commit_message>
working on navigation and adding fa icons
</commit_message>
<xml_diff>
--- a/documentation/table-definitions.xlsx
+++ b/documentation/table-definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repo\Sloth\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78EBC69-85D5-493D-B6E1-8F72E9907FA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC23BE17-06A0-4AC1-978F-B9A301201F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="902" activeTab="7" xr2:uid="{85C21493-8C14-4D37-808F-AD1F9A347F04}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="902" activeTab="1" xr2:uid="{85C21493-8C14-4D37-808F-AD1F9A347F04}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="6" r:id="rId1"/>
@@ -1302,7 +1302,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F0E4785-4EC1-4A2E-A802-88D788D58947}">
   <sheetPr>
-    <tabColor rgb="FFC00000"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1343,7 +1343,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15969139-0295-413B-91FC-574A83A14AD2}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1431,7 +1431,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{231CCF63-9F73-4D4B-8916-53752D386E7D}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1491,7 +1491,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B4235F-3ACD-4C19-A871-E070B0AD7ACB}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1529,7 +1529,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04B9D8C8-7499-425F-8592-AE9E7A39DD51}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1583,7 +1583,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDE1C43D-371D-46C8-B20E-E524A54FD538}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1643,7 +1643,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38CDF530-C106-46D1-B37E-743F829528BC}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1681,7 +1681,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68F4E49F-A596-4E60-832B-44CABE329BB2}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1990,7 +1990,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1C78951-C285-4644-AF28-9C58D430BE32}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2183,7 +2183,7 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F128B1-2C06-41BD-A28F-6E221D2BC9BD}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2287,7 +2287,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0940093-9B6A-4CA7-A81C-636B5D4979ED}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2610,7 +2610,7 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D972206D-678E-4FDE-85FD-45480C65D7ED}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2662,7 +2662,7 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB38038B-DB74-4E09-B26D-28DB8A3D5637}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2757,7 +2757,7 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{234BB3DE-8CFD-4389-98CA-7B40851DC77D}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:R43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2822,7 +2822,7 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05D2246A-D7DF-40CE-9991-016D885B59E4}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2860,7 +2860,7 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB636FF-3550-4F7E-82AC-B6E0EF1AA247}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2946,7 +2946,7 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E9914E-C428-43F5-8933-BAF2D780F56A}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2984,7 +2984,7 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{320490D8-EF2B-4697-B1B6-4928B8A4F0DC}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3022,7 +3022,7 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718E0453-CAF4-43ED-8FF3-A880F2FB1281}">
   <sheetPr>
-    <tabColor theme="8" tint="0.39997558519241921"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3107,7 +3107,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F5E043-9290-49BC-A9A7-B71E9C2E1C9F}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3298,7 +3298,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B2E58E-9AD6-4AB2-940D-895A2CBDA960}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3527,7 +3527,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F275299-BEB8-4E7C-9FD0-238AB3C347C0}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3604,7 +3604,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9353530-2C72-4032-8CA7-97A409477F91}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3861,7 +3861,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E707121-750F-457A-B9B0-13DC5CE04C1F}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4012,7 +4012,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CE7DAE2-49D1-424A-A2C3-097A653826B1}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4201,7 +4201,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE6CD541-770D-4E21-BB1D-83F01DF92677}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>